<commit_message>
Ajoute des identifiants de règle traçables sur chaque suggestion
- Chaque suggestion référence désormais la règle qui l'a produite
  (colonne regle_id dans suggestions.xlsx, exposée en regleId côté API)
- Badge cliquable RG-xx sur chaque carte de suggestion, ouvrant la
  pop-up de règles pré-filtrée et mise en évidence sur la règle visée
- Recherche de la pop-up étendue au code ET à l'identifiant
- 11 règles au total (RG-01 à RG-11, 3 nouvelles pour couvrir fiches/
  observations/mots-clés génériques) : couverture complète des 13
  suggestions du jeu de données de démo
- Chaque règle porte un champ "parametres" structuré (conditions
  {champ, operateur, valeur}) en plus du texte "logique", pensé pour
  être consommé directement par un futur script d'automatisation
- README mis à jour (identifiants, recherche, exemple d'usage de
  "parametres")
</commit_message>
<xml_diff>
--- a/data/suggestions.xlsx
+++ b/data/suggestions.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,6 +479,11 @@
           <t>justification</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>regle_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -529,6 +534,11 @@
           <t>Le terme « cardiopathie ischémique » a été détecté dans le compte-rendu d'hospitalisation.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>RG-04</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -579,6 +589,11 @@
           <t>Mention de « insuffisance rénale aiguë sur chronique stade IIIB » dans le CRH, compatible avec un DFG mesuré à 32-44 mL/min.</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>RG-06</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -629,6 +644,11 @@
           <t>Acte identifié dans le parcours de soins le 05/05 (surveillance diurèse).</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>RG-08</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -679,6 +699,11 @@
           <t>Kaliémie à 3.2-3.4 mmol/L en biologie et mention « kaliémie basse à surveiller » dans le courrier de consultation.</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>RG-07</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -729,6 +754,11 @@
           <t>Aide partielle pour la toilette mentionnée dans la fiche de liaison infirmière.</t>
         </is>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>RG-10</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -779,6 +809,11 @@
           <t>Dyspnée de repos avec orthopnée décrite dans l'observation clinique d'entrée.</t>
         </is>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>RG-11</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -829,6 +864,11 @@
           <t>Pose d'un stent actif mentionnée dans le compte-rendu de coronarographie.</t>
         </is>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>RG-09</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -879,6 +919,11 @@
           <t>Foyer de condensation alvéolaire lobaire décrit sur la radiographie thoracique.</t>
         </is>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>RG-09</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -929,6 +974,11 @@
           <t>Toux productive en diminution mentionnée dans la fiche de surveillance respiratoire.</t>
         </is>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>RG-10</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -979,6 +1029,11 @@
           <t>Pose d'une prothèse totale de hanche mentionnée dans le compte-rendu opératoire.</t>
         </is>
       </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>RG-09</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1029,6 +1084,11 @@
           <t>Hospitalisation programmée pour pose de prothèse de hanche, suggérant une coxarthrose sous-jacente.</t>
         </is>
       </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>RG-09</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1079,6 +1139,11 @@
           <t>Douleur post-opératoire mentionnée dans l'observation clinique du 02/06.</t>
         </is>
       </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>RG-11</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1127,6 +1192,11 @@
       <c r="J14" t="inlineStr">
         <is>
           <t>Coxarthrose évoluée symptomatique mentionnée dans le compte-rendu de consultation.</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>RG-09</t>
         </is>
       </c>
     </row>

</xml_diff>